<commit_message>
update analysis , correlations and fix name bug
</commit_message>
<xml_diff>
--- a/SensitivityAnalysis/data/profile_coeffs_ref.xlsx
+++ b/SensitivityAnalysis/data/profile_coeffs_ref.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Juan\Maestría\Code\oleosim\SensitivityAnalysis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Juan\Maestría\Code\oleosim\SensitivityAnalysis\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A87DFC39-4EDE-42A5-9E3B-5FAAD82BBD89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63B27EFE-418C-450E-A822-8EA6B5926D64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="641" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="641" uniqueCount="83">
   <si>
     <t>Ref</t>
   </si>
@@ -113,9 +113,6 @@
     <t>Linoleic</t>
   </si>
   <si>
-    <t>Plamitic</t>
-  </si>
-  <si>
     <t>Lauric</t>
   </si>
   <si>
@@ -170,9 +167,6 @@
     <t xml:space="preserve">Canola </t>
   </si>
   <si>
-    <t xml:space="preserve">Palm </t>
-  </si>
-  <si>
     <t>Palm - Acid</t>
   </si>
   <si>
@@ -285,6 +279,9 @@
   </si>
   <si>
     <t>20% Beef Tallow - Sunflower</t>
+  </si>
+  <si>
+    <t>Palmitic</t>
   </si>
 </sst>
 </file>
@@ -1212,7 +1209,7 @@
         <v>1</v>
       </c>
       <c r="K15" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
@@ -1247,7 +1244,7 @@
         <v>1</v>
       </c>
       <c r="K16" s="4" t="s">
-        <v>26</v>
+        <v>82</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
@@ -1282,7 +1279,7 @@
         <v>1</v>
       </c>
       <c r="K17" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
@@ -1317,7 +1314,7 @@
         <v>1</v>
       </c>
       <c r="K18" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
@@ -1422,7 +1419,7 @@
         <v>0</v>
       </c>
       <c r="K21" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
@@ -1527,7 +1524,7 @@
         <v>0</v>
       </c>
       <c r="K24" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
@@ -1562,7 +1559,7 @@
         <v>0</v>
       </c>
       <c r="K25" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
@@ -1597,7 +1594,7 @@
         <v>1</v>
       </c>
       <c r="K26" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
@@ -1632,7 +1629,7 @@
         <v>1</v>
       </c>
       <c r="K27" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
@@ -1737,7 +1734,7 @@
         <v>1</v>
       </c>
       <c r="K30" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
@@ -1772,7 +1769,7 @@
         <v>1</v>
       </c>
       <c r="K31" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
@@ -1807,7 +1804,7 @@
         <v>0</v>
       </c>
       <c r="K32" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
@@ -1842,7 +1839,7 @@
         <v>0</v>
       </c>
       <c r="K33" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
@@ -2017,7 +2014,7 @@
         <v>1</v>
       </c>
       <c r="K38" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
@@ -2052,7 +2049,7 @@
         <v>1</v>
       </c>
       <c r="K39" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
@@ -2087,7 +2084,7 @@
         <v>1</v>
       </c>
       <c r="K40" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
@@ -2122,7 +2119,7 @@
         <v>1</v>
       </c>
       <c r="K41" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
@@ -2192,7 +2189,7 @@
         <v>1</v>
       </c>
       <c r="K43" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.25">
@@ -2262,7 +2259,7 @@
         <v>1</v>
       </c>
       <c r="K45" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.25">
@@ -2297,7 +2294,7 @@
         <v>1</v>
       </c>
       <c r="K46" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.25">
@@ -2332,7 +2329,7 @@
         <v>1</v>
       </c>
       <c r="K47" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.25">
@@ -2367,7 +2364,7 @@
         <v>1</v>
       </c>
       <c r="K48" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
@@ -2402,7 +2399,7 @@
         <v>1</v>
       </c>
       <c r="K49" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
@@ -2437,7 +2434,7 @@
         <v>1</v>
       </c>
       <c r="K50" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
@@ -2472,7 +2469,7 @@
         <v>1</v>
       </c>
       <c r="K51" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
@@ -2507,7 +2504,7 @@
         <v>1</v>
       </c>
       <c r="K52" s="4" t="s">
-        <v>45</v>
+        <v>31</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
@@ -2542,7 +2539,7 @@
         <v>1</v>
       </c>
       <c r="K53" s="4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
@@ -2577,7 +2574,7 @@
         <v>1</v>
       </c>
       <c r="K54" s="4" t="s">
-        <v>45</v>
+        <v>31</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
@@ -2612,7 +2609,7 @@
         <v>1</v>
       </c>
       <c r="K55" s="4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
@@ -2647,7 +2644,7 @@
         <v>0</v>
       </c>
       <c r="K56" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
@@ -2682,7 +2679,7 @@
         <v>0</v>
       </c>
       <c r="K57" s="4" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.25">
@@ -2717,7 +2714,7 @@
         <v>0</v>
       </c>
       <c r="K58" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.25">
@@ -2752,7 +2749,7 @@
         <v>0</v>
       </c>
       <c r="K59" s="4" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.25">
@@ -2787,7 +2784,7 @@
         <v>2</v>
       </c>
       <c r="K60" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
@@ -2822,7 +2819,7 @@
         <v>2</v>
       </c>
       <c r="K61" s="4" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.25">
@@ -2857,7 +2854,7 @@
         <v>1</v>
       </c>
       <c r="K62" s="4" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.25">
@@ -2892,7 +2889,7 @@
         <v>1</v>
       </c>
       <c r="K63" s="4" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
@@ -2927,7 +2924,7 @@
         <v>1</v>
       </c>
       <c r="K64" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
@@ -2962,7 +2959,7 @@
         <v>1</v>
       </c>
       <c r="K65" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.25">
@@ -2997,7 +2994,7 @@
         <v>1</v>
       </c>
       <c r="K66" s="4" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
@@ -3032,7 +3029,7 @@
         <v>1</v>
       </c>
       <c r="K67" s="4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
@@ -3067,7 +3064,7 @@
         <v>1</v>
       </c>
       <c r="K68" s="4" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.25">
@@ -3102,7 +3099,7 @@
         <v>1</v>
       </c>
       <c r="K69" s="4" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
@@ -3172,7 +3169,7 @@
         <v>1</v>
       </c>
       <c r="K71" s="4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.25">
@@ -3207,7 +3204,7 @@
         <v>1</v>
       </c>
       <c r="K72" s="4" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
@@ -3242,7 +3239,7 @@
         <v>1</v>
       </c>
       <c r="K73" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
@@ -3277,7 +3274,7 @@
         <v>1</v>
       </c>
       <c r="K74" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
@@ -3312,7 +3309,7 @@
         <v>1</v>
       </c>
       <c r="K75" s="4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.25">
@@ -3382,7 +3379,7 @@
         <v>1</v>
       </c>
       <c r="K77" s="4" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.25">
@@ -3452,7 +3449,7 @@
         <v>1</v>
       </c>
       <c r="K79" s="4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
@@ -3487,7 +3484,7 @@
         <v>1</v>
       </c>
       <c r="K80" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.25">
@@ -3522,7 +3519,7 @@
         <v>1</v>
       </c>
       <c r="K81" s="4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.25">
@@ -3557,7 +3554,7 @@
         <v>1</v>
       </c>
       <c r="K82" s="4" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.25">
@@ -3592,7 +3589,7 @@
         <v>1</v>
       </c>
       <c r="K83" s="4" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.25">
@@ -3627,7 +3624,7 @@
         <v>1</v>
       </c>
       <c r="K84" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.25">
@@ -3662,7 +3659,7 @@
         <v>1</v>
       </c>
       <c r="K85" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.25">
@@ -3697,7 +3694,7 @@
         <v>1</v>
       </c>
       <c r="K86" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="87" spans="1:11" x14ac:dyDescent="0.25">
@@ -3732,7 +3729,7 @@
         <v>1</v>
       </c>
       <c r="K87" s="4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="88" spans="1:11" x14ac:dyDescent="0.25">
@@ -3767,7 +3764,7 @@
         <v>1</v>
       </c>
       <c r="K88" s="4" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="89" spans="1:11" x14ac:dyDescent="0.25">
@@ -3802,7 +3799,7 @@
         <v>1</v>
       </c>
       <c r="K89" s="4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="90" spans="1:11" x14ac:dyDescent="0.25">
@@ -3872,7 +3869,7 @@
         <v>1</v>
       </c>
       <c r="K91" s="4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="92" spans="1:11" x14ac:dyDescent="0.25">
@@ -3907,7 +3904,7 @@
         <v>0</v>
       </c>
       <c r="K92" s="4" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="93" spans="1:11" x14ac:dyDescent="0.25">
@@ -3942,7 +3939,7 @@
         <v>0</v>
       </c>
       <c r="K93" s="4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="94" spans="1:11" x14ac:dyDescent="0.25">
@@ -4082,7 +4079,7 @@
         <v>1</v>
       </c>
       <c r="K97" s="4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="98" spans="1:11" x14ac:dyDescent="0.25">
@@ -4117,7 +4114,7 @@
         <v>1</v>
       </c>
       <c r="K98" s="4" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="99" spans="1:11" x14ac:dyDescent="0.25">
@@ -4152,7 +4149,7 @@
         <v>1</v>
       </c>
       <c r="K99" s="4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="100" spans="1:11" x14ac:dyDescent="0.25">
@@ -4222,7 +4219,7 @@
         <v>1</v>
       </c>
       <c r="K101" s="4" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="102" spans="1:11" x14ac:dyDescent="0.25">
@@ -4257,7 +4254,7 @@
         <v>1</v>
       </c>
       <c r="K102" s="4" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="103" spans="1:11" x14ac:dyDescent="0.25">
@@ -4292,7 +4289,7 @@
         <v>1</v>
       </c>
       <c r="K103" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="104" spans="1:11" x14ac:dyDescent="0.25">
@@ -4327,7 +4324,7 @@
         <v>1</v>
       </c>
       <c r="K104" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="105" spans="1:11" x14ac:dyDescent="0.25">
@@ -4362,7 +4359,7 @@
         <v>1</v>
       </c>
       <c r="K105" s="4" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="106" spans="1:11" x14ac:dyDescent="0.25">
@@ -4397,7 +4394,7 @@
         <v>1</v>
       </c>
       <c r="K106" s="4" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="107" spans="1:11" x14ac:dyDescent="0.25">
@@ -4432,7 +4429,7 @@
         <v>1</v>
       </c>
       <c r="K107" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="108" spans="1:11" x14ac:dyDescent="0.25">
@@ -4467,7 +4464,7 @@
         <v>1</v>
       </c>
       <c r="K108" s="4" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="109" spans="1:11" x14ac:dyDescent="0.25">
@@ -4502,7 +4499,7 @@
         <v>1</v>
       </c>
       <c r="K109" s="4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="110" spans="1:11" x14ac:dyDescent="0.25">
@@ -4572,7 +4569,7 @@
         <v>1</v>
       </c>
       <c r="K111" s="4" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="112" spans="1:11" x14ac:dyDescent="0.25">
@@ -4642,7 +4639,7 @@
         <v>1</v>
       </c>
       <c r="K113" s="4" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="114" spans="1:11" x14ac:dyDescent="0.25">
@@ -4677,7 +4674,7 @@
         <v>1</v>
       </c>
       <c r="K114" s="4" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="115" spans="1:11" x14ac:dyDescent="0.25">
@@ -4712,7 +4709,7 @@
         <v>0</v>
       </c>
       <c r="K115" s="4" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="116" spans="1:11" x14ac:dyDescent="0.25">
@@ -4747,7 +4744,7 @@
         <v>1</v>
       </c>
       <c r="K116" s="4" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="117" spans="1:11" x14ac:dyDescent="0.25">
@@ -4852,7 +4849,7 @@
         <v>1</v>
       </c>
       <c r="K119" s="4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="120" spans="1:11" x14ac:dyDescent="0.25">
@@ -4922,7 +4919,7 @@
         <v>1</v>
       </c>
       <c r="K121" s="4" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="122" spans="1:11" x14ac:dyDescent="0.25">
@@ -4957,7 +4954,7 @@
         <v>1</v>
       </c>
       <c r="K122" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="123" spans="1:11" x14ac:dyDescent="0.25">
@@ -4992,7 +4989,7 @@
         <v>1</v>
       </c>
       <c r="K123" s="4" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="124" spans="1:11" x14ac:dyDescent="0.25">
@@ -5062,7 +5059,7 @@
         <v>0</v>
       </c>
       <c r="K125" s="4" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="126" spans="1:11" x14ac:dyDescent="0.25">
@@ -5097,7 +5094,7 @@
         <v>0</v>
       </c>
       <c r="K126" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="127" spans="1:11" x14ac:dyDescent="0.25">
@@ -5132,7 +5129,7 @@
         <v>1</v>
       </c>
       <c r="K127" s="4" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>